<commit_message>
Add ANOVA validation. Fix T-test after initial validation.
</commit_message>
<xml_diff>
--- a/validation/ttest_data.xlsx
+++ b/validation/ttest_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\t-test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pc\stat_prism\validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80F4B997-0304-4072-BE11-6BE1335D6729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1274FC2-DC92-4049-9249-D5A31D3DD690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,10 +39,10 @@
     <t>Ні</t>
   </si>
   <si>
-    <t>Group</t>
+    <t>Variable Name</t>
   </si>
   <si>
-    <t>Value</t>
+    <t>Group Name</t>
   </si>
 </sst>
 </file>
@@ -339,10 +339,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>